<commit_message>
update labour supply utility to correct vals
</commit_message>
<xml_diff>
--- a/input/reg_labourSupplyUtility.xlsx
+++ b/input/reg_labourSupplyUtility.xlsx
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\andy_local\SimPaths project files\SimPaths\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0B80B9F-6C15-4355-B04D-1D328817DE64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E711D168-67C9-46C7-A4B9-2ABA38379D44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{B28C262A-F414-4C9F-9F20-D497875F2897}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="7" xr2:uid="{B28C262A-F414-4C9F-9F20-D497875F2897}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="8" r:id="rId1"/>
-    <sheet name="UK_Single_Females" sheetId="9" r:id="rId2"/>
-    <sheet name="UK_Single_Males" sheetId="10" r:id="rId3"/>
-    <sheet name="UK_Couples" sheetId="11" r:id="rId4"/>
-    <sheet name="UK_Females_With_Dep" sheetId="12" r:id="rId5"/>
-    <sheet name="UK_Males_With_Dep" sheetId="13" r:id="rId6"/>
-    <sheet name="UK_SingleAC_Females" sheetId="14" r:id="rId7"/>
-    <sheet name="UK_SingleAC_Males" sheetId="15" r:id="rId8"/>
+    <sheet name="UK_Single_Females" sheetId="16" r:id="rId2"/>
+    <sheet name="UK_Single_Males" sheetId="17" r:id="rId3"/>
+    <sheet name="UK_Couples" sheetId="18" r:id="rId4"/>
+    <sheet name="UK_Females_With_Dep" sheetId="19" r:id="rId5"/>
+    <sheet name="UK_Males_With_Dep" sheetId="20" r:id="rId6"/>
+    <sheet name="UK_SingleAC_Females" sheetId="21" r:id="rId7"/>
+    <sheet name="UK_SingleAC_Males" sheetId="22" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="233">
   <si>
     <t>REGRESSOR</t>
   </si>
@@ -438,12 +438,6 @@
     <t>Hrs_36Plus_Male</t>
   </si>
   <si>
-    <t>Hrs_36plus_Male</t>
-  </si>
-  <si>
-    <t>Hrs_36plus_Female</t>
-  </si>
-  <si>
     <t>Liwwh_Male_1</t>
   </si>
   <si>
@@ -684,70 +678,70 @@
     <t>Liwwh_Female_440</t>
   </si>
   <si>
-    <t>Female_Leisure_North_West</t>
+    <t>FemaleLeisure_UKN</t>
   </si>
   <si>
-    <t>Female_Leisure_York_and_Humb</t>
+    <t>FemaleLeisure_UKM</t>
   </si>
   <si>
-    <t>Female_Leisure_East_Mid</t>
+    <t>FemaleLeisure_UKL</t>
   </si>
   <si>
-    <t>Female_Leisure_West_Mid</t>
+    <t>FemaleLeisure_UKK</t>
   </si>
   <si>
-    <t>Female_Leisure_East</t>
+    <t>FemaleLeisure_UKJ</t>
   </si>
   <si>
-    <t>Female_Leisure_London</t>
+    <t>FemaleLeisure_UKI</t>
   </si>
   <si>
-    <t>Female_Leisure_South_East</t>
+    <t>FemaleLeisure_UKH</t>
   </si>
   <si>
-    <t>Female_Leisure_South_West</t>
+    <t>FemaleLeisure_UKG</t>
   </si>
   <si>
-    <t>Female_Leisure_Wales</t>
+    <t>FemaleLeisure_UKF</t>
   </si>
   <si>
-    <t>Female_Leisure_Scotland</t>
+    <t>FemaleLeisure_UKE</t>
   </si>
   <si>
-    <t>Female_Leisure_N_Ireland</t>
+    <t>FemaleLeisure_UKD</t>
   </si>
   <si>
-    <t>Male_Leisure_North_West</t>
+    <t>MaleLeisure_UKN</t>
   </si>
   <si>
-    <t>Male_Leisure_York_and_Humb</t>
+    <t>MaleLeisure_UKM</t>
   </si>
   <si>
-    <t>Male_Leisure_East_Mid</t>
+    <t>MaleLeisure_UKL</t>
   </si>
   <si>
-    <t>Male_Leisure_West_Mid</t>
+    <t>MaleLeisure_UKK</t>
   </si>
   <si>
-    <t>Male_Leisure_East</t>
+    <t>MaleLeisure_UKJ</t>
   </si>
   <si>
-    <t>Male_Leisure_London</t>
+    <t>MaleLeisure_UKI</t>
   </si>
   <si>
-    <t>Male_Leisure_South_East</t>
+    <t>MaleLeisure_UKH</t>
   </si>
   <si>
-    <t>Male_Leisure_South_West</t>
+    <t>MaleLeisure_UKG</t>
   </si>
   <si>
-    <t>Male_Leisure_Wales</t>
+    <t>MaleLeisure_UKF</t>
   </si>
   <si>
-    <t>Male_Leisure_Scotland</t>
+    <t>MaleLeisure_UKE</t>
   </si>
   <si>
-    <t>Male_Leisure_N_Ireland</t>
+    <t>MaleLeisure_UKD</t>
   </si>
 </sst>
 </file>
@@ -1242,11 +1236,12 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A54708F7-E5DF-49D6-BFC9-764EDF2B3988}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2497E15-6FF7-4BEA-8049-BA4982ADFA83}">
   <dimension ref="A1:DD107"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="11.42578125" style="3"/>
+    <col min="1" max="1" width="28.28515625" style="3" customWidth="1"/>
+    <col min="2" max="16384" width="11.42578125" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:108" x14ac:dyDescent="0.25">
@@ -36133,16 +36128,17 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4825F45A-4B0A-410B-A3E0-81D900AD6513}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DB56E65-A028-41C8-8E37-C957AEE6B4E5}">
   <dimension ref="A1:I8"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="11.42578125" style="3"/>
+    <col min="1" max="1" width="39.7109375" style="3" customWidth="1"/>
+    <col min="2" max="16384" width="11.42578125" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -36379,16 +36375,17 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6658EE7-2D33-44C1-A6F2-93177E287D88}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{713A1631-5A78-441A-A83A-D84683700833}">
   <dimension ref="A1:CP93"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="11.42578125" style="3"/>
+    <col min="1" max="1" width="33" style="3" customWidth="1"/>
+    <col min="2" max="16384" width="11.42578125" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:94" x14ac:dyDescent="0.25">
@@ -36429,250 +36426,250 @@
         <v>6</v>
       </c>
       <c r="M1" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="O1" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="W1" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="X1" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="Y1" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="X1" s="3" t="s">
+      <c r="Z1" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="Y1" s="3" t="s">
+      <c r="AA1" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="AB1" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="AA1" s="3" t="s">
+      <c r="AC1" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="AB1" s="3" t="s">
+      <c r="AD1" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="AC1" s="3" t="s">
+      <c r="AE1" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="AD1" s="3" t="s">
+      <c r="AF1" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="AE1" s="3" t="s">
+      <c r="AG1" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="AF1" s="3" t="s">
+      <c r="AH1" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="AG1" s="3" t="s">
+      <c r="AI1" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="AH1" s="3" t="s">
+      <c r="AJ1" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="AI1" s="3" t="s">
+      <c r="AK1" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="AJ1" s="3" t="s">
+      <c r="AL1" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="AK1" s="3" t="s">
+      <c r="AM1" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="AL1" s="3" t="s">
+      <c r="AN1" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="AM1" s="3" t="s">
+      <c r="AO1" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="AN1" s="3" t="s">
+      <c r="AP1" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="AO1" s="3" t="s">
+      <c r="AQ1" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="AP1" s="3" t="s">
+      <c r="AR1" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="AQ1" s="3" t="s">
+      <c r="AS1" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="AR1" s="3" t="s">
+      <c r="AT1" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="AS1" s="3" t="s">
+      <c r="AU1" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="AT1" s="3" t="s">
+      <c r="AV1" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="AU1" s="3" t="s">
+      <c r="AW1" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="AV1" s="3" t="s">
+      <c r="AX1" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="AW1" s="3" t="s">
+      <c r="AY1" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="AX1" s="3" t="s">
+      <c r="AZ1" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="AY1" s="3" t="s">
+      <c r="BA1" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="AZ1" s="3" t="s">
+      <c r="BB1" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="BA1" s="3" t="s">
+      <c r="BC1" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="BB1" s="3" t="s">
+      <c r="BD1" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="BC1" s="3" t="s">
+      <c r="BE1" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="BD1" s="3" t="s">
+      <c r="BF1" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="BE1" s="3" t="s">
+      <c r="BG1" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="BF1" s="3" t="s">
+      <c r="BH1" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="BG1" s="3" t="s">
+      <c r="BI1" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="BH1" s="3" t="s">
+      <c r="BJ1" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="BI1" s="3" t="s">
+      <c r="BK1" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="BJ1" s="3" t="s">
+      <c r="BL1" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="BK1" s="3" t="s">
+      <c r="BM1" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="BL1" s="3" t="s">
+      <c r="BN1" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="BM1" s="3" t="s">
+      <c r="BO1" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="BN1" s="3" t="s">
+      <c r="BP1" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="BO1" s="3" t="s">
+      <c r="BQ1" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="BP1" s="3" t="s">
+      <c r="BR1" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="BQ1" s="3" t="s">
+      <c r="BS1" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="BR1" s="3" t="s">
+      <c r="BT1" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="BS1" s="3" t="s">
+      <c r="BU1" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="BT1" s="3" t="s">
+      <c r="BV1" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="BU1" s="3" t="s">
+      <c r="BW1" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="BV1" s="3" t="s">
+      <c r="BX1" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="BW1" s="3" t="s">
+      <c r="BY1" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="BX1" s="3" t="s">
+      <c r="BZ1" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="BY1" s="3" t="s">
+      <c r="CA1" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="BZ1" s="3" t="s">
+      <c r="CB1" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="CA1" s="3" t="s">
+      <c r="CC1" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="CB1" s="3" t="s">
+      <c r="CD1" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="CC1" s="3" t="s">
+      <c r="CE1" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="CD1" s="3" t="s">
+      <c r="CF1" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="CE1" s="3" t="s">
+      <c r="CG1" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="CF1" s="3" t="s">
+      <c r="CH1" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="CG1" s="3" t="s">
+      <c r="CI1" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="CH1" s="3" t="s">
+      <c r="CJ1" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="CI1" s="3" t="s">
+      <c r="CK1" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="CJ1" s="3" t="s">
+      <c r="CL1" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="CK1" s="3" t="s">
+      <c r="CM1" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="CL1" s="3" t="s">
+      <c r="CN1" s="3" t="s">
         <v>208</v>
       </c>
-      <c r="CM1" s="3" t="s">
+      <c r="CO1" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="CN1" s="3" t="s">
+      <c r="CP1" s="3" t="s">
         <v>210</v>
-      </c>
-      <c r="CO1" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="CP1" s="3" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:94" x14ac:dyDescent="0.25">
@@ -40085,7 +40082,7 @@
     </row>
     <row r="14" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B14" s="3">
         <v>-0.24851257653206699</v>
@@ -40369,7 +40366,7 @@
     </row>
     <row r="15" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B15" s="3">
         <v>-0.15501650152683599</v>
@@ -40653,7 +40650,7 @@
     </row>
     <row r="16" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B16" s="3">
         <v>-3.3557569295545202E-2</v>
@@ -40937,7 +40934,7 @@
     </row>
     <row r="17" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B17" s="3">
         <v>3.1086688130075299E-2</v>
@@ -41221,7 +41218,7 @@
     </row>
     <row r="18" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B18" s="3">
         <v>-3.54804655910477E-2</v>
@@ -41505,7 +41502,7 @@
     </row>
     <row r="19" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B19" s="3">
         <v>0.104490784522007</v>
@@ -41789,7 +41786,7 @@
     </row>
     <row r="20" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B20" s="3">
         <v>-1.6740910505204602E-2</v>
@@ -42073,7 +42070,7 @@
     </row>
     <row r="21" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B21" s="3">
         <v>2.68411381805354E-2</v>
@@ -42357,7 +42354,7 @@
     </row>
     <row r="22" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B22" s="3">
         <v>3.9140421628870901E-2</v>
@@ -42641,7 +42638,7 @@
     </row>
     <row r="23" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B23" s="3">
         <v>3.6009585048853501E-2</v>
@@ -42925,7 +42922,7 @@
     </row>
     <row r="24" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B24" s="3">
         <v>-4.1153464270304002E-2</v>
@@ -43209,7 +43206,7 @@
     </row>
     <row r="25" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B25" s="3">
         <v>5.2805973843852799E-2</v>
@@ -43493,7 +43490,7 @@
     </row>
     <row r="26" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B26" s="3">
         <v>-0.24664046507380399</v>
@@ -43777,7 +43774,7 @@
     </row>
     <row r="27" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B27" s="3">
         <v>-8.16818341777997E-2</v>
@@ -44061,7 +44058,7 @@
     </row>
     <row r="28" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B28" s="3">
         <v>-2.7376636525575999E-2</v>
@@ -44345,7 +44342,7 @@
     </row>
     <row r="29" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B29" s="3">
         <v>3.6859599206483303E-2</v>
@@ -44629,7 +44626,7 @@
     </row>
     <row r="30" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B30" s="3">
         <v>-0.266921014426866</v>
@@ -44913,7 +44910,7 @@
     </row>
     <row r="31" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B31" s="3">
         <v>-9.4004542275197001E-2</v>
@@ -45197,7 +45194,7 @@
     </row>
     <row r="32" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B32" s="3">
         <v>-1.28983256881103E-2</v>
@@ -45481,7 +45478,7 @@
     </row>
     <row r="33" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B33" s="3">
         <v>1.39806666058512E-2</v>
@@ -45765,7 +45762,7 @@
     </row>
     <row r="34" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B34" s="3">
         <v>-0.241530621994761</v>
@@ -46049,7 +46046,7 @@
     </row>
     <row r="35" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B35" s="3">
         <v>-0.147615297043832</v>
@@ -46333,7 +46330,7 @@
     </row>
     <row r="36" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B36" s="3">
         <v>-3.0341143642342298E-2</v>
@@ -46617,7 +46614,7 @@
     </row>
     <row r="37" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B37" s="3">
         <v>3.07085183522318E-2</v>
@@ -46901,7 +46898,7 @@
     </row>
     <row r="38" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B38" s="3">
         <v>-0.235620706291398</v>
@@ -47185,7 +47182,7 @@
     </row>
     <row r="39" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B39" s="3">
         <v>-0.14108344291893599</v>
@@ -47469,7 +47466,7 @@
     </row>
     <row r="40" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B40" s="3">
         <v>-3.1069493186529198E-2</v>
@@ -47753,7 +47750,7 @@
     </row>
     <row r="41" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B41" s="3">
         <v>4.4659950017029999E-2</v>
@@ -48037,7 +48034,7 @@
     </row>
     <row r="42" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B42" s="3">
         <v>-0.25460426377618001</v>
@@ -48321,7 +48318,7 @@
     </row>
     <row r="43" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B43" s="3">
         <v>-8.3970811896098896E-2</v>
@@ -48605,7 +48602,7 @@
     </row>
     <row r="44" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B44" s="3">
         <v>-2.3993425911259199E-2</v>
@@ -48889,7 +48886,7 @@
     </row>
     <row r="45" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B45" s="3">
         <v>4.06632647854046E-2</v>
@@ -49173,7 +49170,7 @@
     </row>
     <row r="46" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B46" s="3">
         <v>-0.245869225848625</v>
@@ -49457,7 +49454,7 @@
     </row>
     <row r="47" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B47" s="3">
         <v>-8.1010365828426203E-2</v>
@@ -49741,7 +49738,7 @@
     </row>
     <row r="48" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B48" s="3">
         <v>-2.7620053894158701E-2</v>
@@ -50025,7 +50022,7 @@
     </row>
     <row r="49" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B49" s="3">
         <v>3.3648476392357199E-2</v>
@@ -50309,7 +50306,7 @@
     </row>
     <row r="50" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B50" s="3">
         <v>-0.27974082537358902</v>
@@ -50593,7 +50590,7 @@
     </row>
     <row r="51" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B51" s="3">
         <v>-7.9125985712695704E-2</v>
@@ -50877,7 +50874,7 @@
     </row>
     <row r="52" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B52" s="3">
         <v>1.16923849670512E-2</v>
@@ -51161,7 +51158,7 @@
     </row>
     <row r="53" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B53" s="3">
         <v>-2.37213448911E-3</v>
@@ -51445,7 +51442,7 @@
     </row>
     <row r="54" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B54" s="3">
         <v>-0.23817014524878</v>
@@ -51729,7 +51726,7 @@
     </row>
     <row r="55" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B55" s="3">
         <v>-0.143863760962225</v>
@@ -52013,7 +52010,7 @@
     </row>
     <row r="56" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B56" s="3">
         <v>-1.9193132946093001E-2</v>
@@ -52297,7 +52294,7 @@
     </row>
     <row r="57" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B57" s="3">
         <v>2.9104616195848799E-2</v>
@@ -52581,7 +52578,7 @@
     </row>
     <row r="58" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B58" s="3">
         <v>-0.26222573600960403</v>
@@ -52865,7 +52862,7 @@
     </row>
     <row r="59" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B59" s="3">
         <v>-8.7324478884078599E-2</v>
@@ -53149,7 +53146,7 @@
     </row>
     <row r="60" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B60" s="3">
         <v>-8.0538958530602008E-3</v>
@@ -53433,7 +53430,7 @@
     </row>
     <row r="61" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B61" s="3">
         <v>3.4468551042118899E-2</v>
@@ -53717,7 +53714,7 @@
     </row>
     <row r="62" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B62" s="3">
         <v>-5.8149600710401704E-3</v>
@@ -54001,7 +53998,7 @@
     </row>
     <row r="63" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B63" s="3">
         <v>3.2403465051017197E-2</v>
@@ -54285,7 +54282,7 @@
     </row>
     <row r="64" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B64" s="3">
         <v>-1.95968544991071E-2</v>
@@ -54569,7 +54566,7 @@
     </row>
     <row r="65" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B65" s="3">
         <v>4.3088570435007703E-2</v>
@@ -54853,7 +54850,7 @@
     </row>
     <row r="66" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B66" s="3">
         <v>1.3782593123408699E-2</v>
@@ -55137,7 +55134,7 @@
     </row>
     <row r="67" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B67" s="3">
         <v>4.2217819515446E-3</v>
@@ -55421,7 +55418,7 @@
     </row>
     <row r="68" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B68" s="3">
         <v>-0.24101550673286201</v>
@@ -55705,7 +55702,7 @@
     </row>
     <row r="69" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B69" s="3">
         <v>-0.14407589532802201</v>
@@ -55989,7 +55986,7 @@
     </row>
     <row r="70" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B70" s="3">
         <v>-1.37294896327869E-2</v>
@@ -56273,7 +56270,7 @@
     </row>
     <row r="71" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B71" s="3">
         <v>3.73680753415431E-2</v>
@@ -56557,7 +56554,7 @@
     </row>
     <row r="72" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B72" s="3">
         <v>-0.26682852387940398</v>
@@ -56841,7 +56838,7 @@
     </row>
     <row r="73" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B73" s="3">
         <v>-8.8436226125812104E-2</v>
@@ -57125,7 +57122,7 @@
     </row>
     <row r="74" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B74" s="3">
         <v>6.8005805226868698E-4</v>
@@ -57409,7 +57406,7 @@
     </row>
     <row r="75" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B75" s="3">
         <v>3.3848348666552203E-2</v>
@@ -57693,7 +57690,7 @@
     </row>
     <row r="76" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B76" s="3">
         <v>-8.8371173287494901E-4</v>
@@ -57977,7 +57974,7 @@
     </row>
     <row r="77" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B77" s="3">
         <v>4.04919256273501E-2</v>
@@ -58261,7 +58258,7 @@
     </row>
     <row r="78" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B78" s="3">
         <v>-1.24503691831E-2</v>
@@ -58545,7 +58542,7 @@
     </row>
     <row r="79" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B79" s="3">
         <v>4.4795385372791097E-2</v>
@@ -58829,7 +58826,7 @@
     </row>
     <row r="80" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B80" s="3">
         <v>2.0286667152899299E-3</v>
@@ -59113,7 +59110,7 @@
     </row>
     <row r="81" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B81" s="3">
         <v>3.6560329427985602E-3</v>
@@ -59397,7 +59394,7 @@
     </row>
     <row r="82" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B82" s="3">
         <v>7.0307314940585106E-2</v>
@@ -59681,7 +59678,7 @@
     </row>
     <row r="83" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B83" s="3">
         <v>-1.33212316156076</v>
@@ -59965,7 +59962,7 @@
     </row>
     <row r="84" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B84" s="3">
         <v>-8.9552728282690404E-3</v>
@@ -60249,7 +60246,7 @@
     </row>
     <row r="85" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B85" s="3">
         <v>1.9935071355956201E-2</v>
@@ -60533,7 +60530,7 @@
     </row>
     <row r="86" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B86" s="3">
         <v>-0.28281924164622801</v>
@@ -60817,7 +60814,7 @@
     </row>
     <row r="87" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B87" s="3">
         <v>-9.6856980827706898E-2</v>
@@ -61101,7 +61098,7 @@
     </row>
     <row r="88" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B88" s="3">
         <v>-1.0029218489704599E-2</v>
@@ -61385,7 +61382,7 @@
     </row>
     <row r="89" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B89" s="3">
         <v>3.4912659661339801E-2</v>
@@ -61669,7 +61666,7 @@
     </row>
     <row r="90" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B90" s="3">
         <v>-6.8797262004654299E-3</v>
@@ -61953,7 +61950,7 @@
     </row>
     <row r="91" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B91" s="3">
         <v>3.8238204748118503E-2</v>
@@ -62237,7 +62234,7 @@
     </row>
     <row r="92" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B92" s="3">
         <v>-1.19181161641839E-2</v>
@@ -62521,7 +62518,7 @@
     </row>
     <row r="93" spans="1:94" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B93" s="3">
         <v>3.7717663714500901E-2</v>
@@ -62805,16 +62802,17 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9416BC3F-8B82-4765-A088-74681707CDEE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A52A53A-8337-4C79-8847-E5AFC5268D50}">
   <dimension ref="A1:I8"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="11.42578125" style="3"/>
+    <col min="1" max="1" width="33.42578125" style="3" customWidth="1"/>
+    <col min="2" max="16384" width="11.42578125" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -63051,16 +63049,17 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09372B0C-F30D-4D98-96DC-582249BCF77D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9164393-5E7D-4422-9A61-B7FFE1623344}">
   <dimension ref="A1:I8"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="11.42578125" style="3"/>
+    <col min="1" max="1" width="30" style="3" customWidth="1"/>
+    <col min="2" max="16384" width="11.42578125" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -63297,16 +63296,17 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0FB52BB-C20E-4BC6-976E-47599FA26233}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46DFF46C-488E-4562-9683-A336EF32C45A}">
   <dimension ref="A1:T19"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="11.42578125" style="3"/>
+    <col min="1" max="1" width="46.140625" style="3" customWidth="1"/>
+    <col min="2" max="16384" width="11.42578125" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -63338,37 +63338,37 @@
         <v>29</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="N1" s="3" t="s">
         <v>217</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="Q1" s="3" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="R1" s="3" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="S1" s="3" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
       <c r="T1" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
@@ -63807,7 +63807,7 @@
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="B9" s="3">
         <v>-8.1972965338796E-3</v>
@@ -63869,7 +63869,7 @@
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="B10" s="3">
         <v>-6.8212570985156198E-4</v>
@@ -63931,7 +63931,7 @@
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="B11" s="3">
         <v>-4.4596424160110298E-4</v>
@@ -63993,7 +63993,7 @@
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B12" s="3">
         <v>-5.4173523046E-3</v>
@@ -64117,7 +64117,7 @@
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B14" s="3">
         <v>7.0813954923913802E-3</v>
@@ -64179,7 +64179,7 @@
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="B15" s="3">
         <v>-8.6466993167642007E-3</v>
@@ -64241,7 +64241,7 @@
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="B16" s="3">
         <v>-1.52704841429614E-2</v>
@@ -64303,7 +64303,7 @@
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="B17" s="3">
         <v>6.8823809369989702E-3</v>
@@ -64365,7 +64365,7 @@
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
       <c r="B18" s="3">
         <v>-1.56186443086244E-2</v>
@@ -64427,7 +64427,7 @@
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="B19" s="3">
         <v>-1.07160697847995E-2</v>
@@ -64489,16 +64489,17 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F9CCDAC-EBCE-4616-82D5-20E839EE650F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DFE8567-67A3-41A3-9804-ADC448CEC0EA}">
   <dimension ref="A1:T19"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="11.42578125" style="3"/>
+    <col min="1" max="1" width="32.140625" style="3" customWidth="1"/>
+    <col min="2" max="16384" width="11.42578125" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -64530,37 +64531,37 @@
         <v>130</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="N1" s="3" t="s">
         <v>228</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="Q1" s="3" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="R1" s="3" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="S1" s="3" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="T1" s="3" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
@@ -64999,7 +65000,7 @@
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="B9" s="3">
         <v>-8.1972965338796E-3</v>
@@ -65061,7 +65062,7 @@
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="B10" s="3">
         <v>-6.8212570985156198E-4</v>
@@ -65123,7 +65124,7 @@
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="B11" s="3">
         <v>-4.4596424160110298E-4</v>
@@ -65185,7 +65186,7 @@
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B12" s="3">
         <v>-5.4173523046E-3</v>
@@ -65309,7 +65310,7 @@
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="B14" s="3">
         <v>7.0813954923913802E-3</v>
@@ -65371,7 +65372,7 @@
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="B15" s="3">
         <v>-8.6466993167642007E-3</v>
@@ -65433,7 +65434,7 @@
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="B16" s="3">
         <v>-1.52704841429614E-2</v>
@@ -65495,7 +65496,7 @@
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="B17" s="3">
         <v>6.8823809369989702E-3</v>
@@ -65557,7 +65558,7 @@
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="B18" s="3">
         <v>-1.56186443086244E-2</v>
@@ -65619,7 +65620,7 @@
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="B19" s="3">
         <v>-1.07160697847995E-2</v>
@@ -65681,6 +65682,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>